<commit_message>
Add visible cell borders to the answer form so rows are easy to track
</commit_message>
<xml_diff>
--- a/Jeopardy Answer Form.xlsx
+++ b/Jeopardy Answer Form.xlsx
@@ -80,7 +80,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -88,11 +88,25 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00B7BFD1"/>
+      </left>
+      <right style="thin">
+        <color rgb="00B7BFD1"/>
+      </right>
+      <top style="thin">
+        <color rgb="00B7BFD1"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00B7BFD1"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -101,17 +115,16 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -578,12 +591,12 @@
       <c r="B2" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C2" s="7" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Name the locations of your first 3 dates</t>
         </is>
       </c>
-      <c r="D2" s="8" t="inlineStr"/>
+      <c r="D2" s="7" t="inlineStr"/>
     </row>
     <row r="3" ht="30" customHeight="1">
       <c r="A3" s="5" t="inlineStr">
@@ -594,12 +607,12 @@
       <c r="B3" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Who said “I love you” first, and when?</t>
         </is>
       </c>
-      <c r="D3" s="8" t="inlineStr"/>
+      <c r="D3" s="7" t="inlineStr"/>
     </row>
     <row r="4" ht="30" customHeight="1">
       <c r="A4" s="5" t="inlineStr">
@@ -610,12 +623,12 @@
       <c r="B4" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="C4" s="7" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>When do you think you knew you were going to marry your fiancé?</t>
         </is>
       </c>
-      <c r="D4" s="8" t="inlineStr"/>
+      <c r="D4" s="7" t="inlineStr"/>
     </row>
     <row r="5" ht="30" customHeight="1">
       <c r="A5" s="5" t="inlineStr">
@@ -626,12 +639,12 @@
       <c r="B5" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>What is the first thing your fiancé said after the proposal?</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr"/>
+      <c r="D5" s="7" t="inlineStr"/>
     </row>
     <row r="6" ht="30" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
@@ -642,8 +655,8 @@
       <c r="B6" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="C6" s="7" t="inlineStr"/>
-      <c r="D6" s="8" t="inlineStr"/>
+      <c r="C6" s="5" t="inlineStr"/>
+      <c r="D6" s="7" t="inlineStr"/>
     </row>
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
@@ -654,12 +667,12 @@
       <c r="B7" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>What is one thing your fiancé can’t live without?</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr"/>
+      <c r="D7" s="7" t="inlineStr"/>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
@@ -670,12 +683,12 @@
       <c r="B8" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="C8" s="7" t="inlineStr">
+      <c r="C8" s="5" t="inlineStr">
         <is>
           <t>What do you find most attractive about your fiancé?</t>
         </is>
       </c>
-      <c r="D8" s="8" t="inlineStr"/>
+      <c r="D8" s="7" t="inlineStr"/>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
@@ -686,12 +699,12 @@
       <c r="B9" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>What superhero would your fiancé be, and why?</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
@@ -702,12 +715,12 @@
       <c r="B10" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="C10" s="7" t="inlineStr">
+      <c r="C10" s="5" t="inlineStr">
         <is>
           <t>What is your fiancé’s idea of a perfect date?</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="5" t="inlineStr">
@@ -718,12 +731,12 @@
       <c r="B11" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>What is your fiancé most excited about for the wedding?</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr"/>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
@@ -734,12 +747,12 @@
       <c r="B12" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C12" s="7" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>What is one thing you can’t live without?</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr"/>
+      <c r="D12" s="7" t="inlineStr"/>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="5" t="inlineStr">
@@ -750,12 +763,12 @@
       <c r="B13" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="5" t="inlineStr">
         <is>
           <t>What superhero would you be, and why?</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr"/>
+      <c r="D13" s="7" t="inlineStr"/>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="5" t="inlineStr">
@@ -766,12 +779,12 @@
       <c r="B14" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="C14" s="7" t="inlineStr">
+      <c r="C14" s="5" t="inlineStr">
         <is>
           <t>What is your idea of a perfect date?</t>
         </is>
       </c>
-      <c r="D14" s="8" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr"/>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="5" t="inlineStr">
@@ -782,12 +795,12 @@
       <c r="B15" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>What are you most excited about for the wedding?</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr"/>
+      <c r="D15" s="7" t="inlineStr"/>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="5" t="inlineStr">
@@ -798,8 +811,8 @@
       <c r="B16" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="C16" s="7" t="inlineStr"/>
-      <c r="D16" s="8" t="inlineStr"/>
+      <c r="C16" s="5" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr"/>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="5" t="inlineStr">
@@ -810,12 +823,12 @@
       <c r="B17" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="5" t="inlineStr">
         <is>
           <t>What would your fiancé get rid of in your closet?</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr"/>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="5" t="inlineStr">
@@ -826,12 +839,12 @@
       <c r="B18" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>What would you get rid of in your fiancé’s closet?</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr"/>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="5" t="inlineStr">
@@ -842,12 +855,12 @@
       <c r="B19" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>What is one thing you do that annoys your fiancé the most?</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr"/>
+      <c r="D19" s="7" t="inlineStr"/>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
@@ -858,12 +871,12 @@
       <c r="B20" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="C20" s="7" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>What is one thing your fiancé does that annoys you the most?</t>
         </is>
       </c>
-      <c r="D20" s="8" t="inlineStr"/>
+      <c r="D20" s="7" t="inlineStr"/>
     </row>
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="5" t="inlineStr">
@@ -874,8 +887,8 @@
       <c r="B21" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="C21" s="7" t="inlineStr"/>
-      <c r="D21" s="8" t="inlineStr"/>
+      <c r="C21" s="5" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr"/>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
@@ -886,12 +899,12 @@
       <c r="B22" s="6" t="n">
         <v>200</v>
       </c>
-      <c r="C22" s="7" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>What is the last concert/event you went to together?</t>
         </is>
       </c>
-      <c r="D22" s="8" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr"/>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="5" t="inlineStr">
@@ -902,12 +915,12 @@
       <c r="B23" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>What is the most memorable meal you shared?</t>
         </is>
       </c>
-      <c r="D23" s="8" t="inlineStr"/>
+      <c r="D23" s="7" t="inlineStr"/>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="5" t="inlineStr">
@@ -918,8 +931,8 @@
       <c r="B24" s="6" t="n">
         <v>600</v>
       </c>
-      <c r="C24" s="7" t="inlineStr"/>
-      <c r="D24" s="8" t="inlineStr"/>
+      <c r="C24" s="5" t="inlineStr"/>
+      <c r="D24" s="7" t="inlineStr"/>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
@@ -930,8 +943,8 @@
       <c r="B25" s="6" t="n">
         <v>800</v>
       </c>
-      <c r="C25" s="7" t="inlineStr"/>
-      <c r="D25" s="8" t="inlineStr"/>
+      <c r="C25" s="5" t="inlineStr"/>
+      <c r="D25" s="7" t="inlineStr"/>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="5" t="inlineStr">
@@ -942,8 +955,8 @@
       <c r="B26" s="6" t="n">
         <v>1000</v>
       </c>
-      <c r="C26" s="7" t="inlineStr"/>
-      <c r="D26" s="8" t="inlineStr"/>
+      <c r="C26" s="5" t="inlineStr"/>
+      <c r="D26" s="7" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>